<commit_message>
changed Romania profile Moderate risk (mixed) to Moderate substance use same changes applied to hbsc_labels.xlsx and profile mapping in the webapp
</commit_message>
<xml_diff>
--- a/data/hbsc_labels.xlsx
+++ b/data/hbsc_labels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hanst\.rstudio\projects\Bechtiger &amp; Janousch (2025) Adolescent Well-Being in Flux\Adolescent-Well-Being-in-Flux\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C818308-3CFF-4CF6-AA68-2C6DF2F7BFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26099BAC-5934-499A-B312-E17E0238B5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3021" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3021" uniqueCount="108">
   <si>
     <t>Country</t>
   </si>
@@ -359,9 +359,6 @@
   </si>
   <si>
     <t>Mixed moderate risk</t>
-  </si>
-  <si>
-    <t>Moderate risk (mixed)</t>
   </si>
   <si>
     <t>Highest risk</t>
@@ -1035,13 +1032,13 @@
         <v>73</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
         <v>78</v>
       </c>
       <c r="W2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X2" t="s">
         <v>78</v>
@@ -1050,7 +1047,7 @@
         <v>78</v>
       </c>
       <c r="AC2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.45">
@@ -1067,10 +1064,10 @@
         <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S3" t="s">
         <v>84</v>
@@ -1079,7 +1076,7 @@
         <v>78</v>
       </c>
       <c r="W3" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X3" t="s">
         <v>78</v>
@@ -1094,7 +1091,7 @@
         <v>84</v>
       </c>
       <c r="AD3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.45">
@@ -1108,7 +1105,7 @@
         <v>78</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E4" t="s">
         <v>86</v>
@@ -1120,7 +1117,7 @@
         <v>85</v>
       </c>
       <c r="I4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J4" t="s">
         <v>84</v>
@@ -1135,7 +1132,7 @@
         <v>85</v>
       </c>
       <c r="O4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P4" t="s">
         <v>84</v>
@@ -1150,10 +1147,10 @@
         <v>85</v>
       </c>
       <c r="U4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X4" t="s">
         <v>85</v>
@@ -1165,7 +1162,7 @@
         <v>89</v>
       </c>
       <c r="AB4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC4" t="s">
         <v>86</v>
@@ -1185,7 +1182,7 @@
         <v>74</v>
       </c>
       <c r="C5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s">
         <v>84</v>
@@ -1194,7 +1191,7 @@
         <v>78</v>
       </c>
       <c r="AB5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC5" t="s">
         <v>84</v>
@@ -1220,7 +1217,7 @@
         <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H6" t="s">
         <v>85</v>
@@ -1232,10 +1229,10 @@
         <v>78</v>
       </c>
       <c r="K6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N6" t="s">
         <v>78</v>
@@ -1250,7 +1247,7 @@
         <v>78</v>
       </c>
       <c r="S6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T6" t="s">
         <v>84</v>
@@ -1268,13 +1265,13 @@
         <v>84</v>
       </c>
       <c r="Z6" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB6" s="30" t="s">
         <v>86</v>
       </c>
       <c r="AC6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD6" t="s">
         <v>78</v>
@@ -1294,7 +1291,7 @@
         <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E7" t="s">
         <v>86</v>
@@ -1311,7 +1308,7 @@
         <v>78</v>
       </c>
       <c r="O7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P7" t="s">
         <v>85</v>
@@ -1323,7 +1320,7 @@
         <v>84</v>
       </c>
       <c r="T7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U7" t="s">
         <v>85</v>
@@ -1332,7 +1329,7 @@
         <v>78</v>
       </c>
       <c r="X7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y7" t="s">
         <v>86</v>
@@ -1350,7 +1347,7 @@
         <v>78</v>
       </c>
       <c r="AE7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.45">
@@ -1361,7 +1358,7 @@
         <v>75</v>
       </c>
       <c r="C8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
         <v>86</v>
@@ -1376,7 +1373,7 @@
         <v>85</v>
       </c>
       <c r="N8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O8" t="s">
         <v>78</v>
@@ -1388,7 +1385,7 @@
         <v>78</v>
       </c>
       <c r="X8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y8" t="s">
         <v>85</v>
@@ -1400,7 +1397,7 @@
         <v>78</v>
       </c>
       <c r="AC8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD8" s="29" t="s">
         <v>86</v>
@@ -1423,13 +1420,13 @@
         <v>85</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
         <v>78</v>
       </c>
       <c r="I9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J9" t="s">
         <v>85</v>
@@ -1441,10 +1438,10 @@
         <v>78</v>
       </c>
       <c r="O9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R9" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S9" t="s">
         <v>78</v>
@@ -1456,7 +1453,7 @@
         <v>78</v>
       </c>
       <c r="X9" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y9" t="s">
         <v>85</v>
@@ -1468,7 +1465,7 @@
         <v>78</v>
       </c>
       <c r="AD9" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.45">
@@ -1482,7 +1479,7 @@
         <v>78</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E10" t="s">
         <v>85</v>
@@ -1494,7 +1491,7 @@
         <v>84</v>
       </c>
       <c r="I10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J10" t="s">
         <v>85</v>
@@ -1503,7 +1500,7 @@
         <v>78</v>
       </c>
       <c r="M10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N10" t="s">
         <v>84</v>
@@ -1515,7 +1512,7 @@
         <v>85</v>
       </c>
       <c r="R10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S10" t="s">
         <v>78</v>
@@ -1527,7 +1524,7 @@
         <v>85</v>
       </c>
       <c r="W10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X10" t="s">
         <v>86</v>
@@ -1548,7 +1545,7 @@
         <v>78</v>
       </c>
       <c r="AE10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.45">
@@ -1568,7 +1565,7 @@
         <v>78</v>
       </c>
       <c r="F11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H11" t="s">
         <v>84</v>
@@ -1577,13 +1574,13 @@
         <v>78</v>
       </c>
       <c r="J11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K11" t="s">
         <v>85</v>
       </c>
       <c r="M11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N11" t="s">
         <v>84</v>
@@ -1598,7 +1595,7 @@
         <v>85</v>
       </c>
       <c r="S11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T11" t="s">
         <v>78</v>
@@ -1616,7 +1613,7 @@
         <v>85</v>
       </c>
       <c r="Z11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB11" t="s">
         <v>78</v>
@@ -1628,7 +1625,7 @@
         <v>86</v>
       </c>
       <c r="AE11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.45">
@@ -1645,7 +1642,7 @@
         <v>78</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H12" t="s">
         <v>85</v>
@@ -1654,7 +1651,7 @@
         <v>78</v>
       </c>
       <c r="J12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M12" t="s">
         <v>78</v>
@@ -1663,7 +1660,7 @@
         <v>85</v>
       </c>
       <c r="O12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R12" t="s">
         <v>78</v>
@@ -1672,7 +1669,7 @@
         <v>85</v>
       </c>
       <c r="T12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W12" t="s">
         <v>78</v>
@@ -1681,13 +1678,13 @@
         <v>85</v>
       </c>
       <c r="Y12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB12" t="s">
         <v>85</v>
       </c>
       <c r="AC12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD12" t="s">
         <v>78</v>
@@ -1701,7 +1698,7 @@
         <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
         <v>78</v>
@@ -1716,10 +1713,10 @@
         <v>78</v>
       </c>
       <c r="J13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N13" t="s">
         <v>78</v>
@@ -1731,7 +1728,7 @@
         <v>78</v>
       </c>
       <c r="S13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T13" t="s">
         <v>85</v>
@@ -1743,13 +1740,13 @@
         <v>78</v>
       </c>
       <c r="Y13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB13" t="s">
         <v>78</v>
       </c>
       <c r="AC13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD13" t="s">
         <v>86</v>
@@ -1766,7 +1763,7 @@
         <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E14" t="s">
         <v>86</v>
@@ -1781,7 +1778,7 @@
         <v>85</v>
       </c>
       <c r="J14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K14" t="s">
         <v>84</v>
@@ -1793,7 +1790,7 @@
         <v>78</v>
       </c>
       <c r="O14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P14" t="s">
         <v>85</v>
@@ -1808,7 +1805,7 @@
         <v>85</v>
       </c>
       <c r="U14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W14" t="s">
         <v>78</v>
@@ -1817,7 +1814,7 @@
         <v>84</v>
       </c>
       <c r="Y14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Z14" t="s">
         <v>85</v>
@@ -1829,7 +1826,7 @@
         <v>78</v>
       </c>
       <c r="AD14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE14" t="s">
         <v>85</v>
@@ -1852,7 +1849,7 @@
         <v>78</v>
       </c>
       <c r="F15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H15" t="s">
         <v>85</v>
@@ -1864,7 +1861,7 @@
         <v>78</v>
       </c>
       <c r="K15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M15" t="s">
         <v>89</v>
@@ -1873,7 +1870,7 @@
         <v>85</v>
       </c>
       <c r="O15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P15" t="s">
         <v>78</v>
@@ -1888,7 +1885,7 @@
         <v>84</v>
       </c>
       <c r="U15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W15" t="s">
         <v>85</v>
@@ -1900,10 +1897,10 @@
         <v>78</v>
       </c>
       <c r="Z15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC15" t="s">
         <v>78</v>
@@ -1923,7 +1920,7 @@
         <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
         <v>85</v>
@@ -1938,10 +1935,10 @@
         <v>85</v>
       </c>
       <c r="J16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N16" t="s">
         <v>78</v>
@@ -1956,10 +1953,10 @@
         <v>85</v>
       </c>
       <c r="T16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X16" t="s">
         <v>85</v>
@@ -1974,7 +1971,7 @@
         <v>78</v>
       </c>
       <c r="AD16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.45">
@@ -1985,13 +1982,13 @@
         <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D17" t="s">
         <v>78</v>
       </c>
       <c r="AB17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC17" t="s">
         <v>78</v>
@@ -2014,7 +2011,7 @@
         <v>78</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H18" t="s">
         <v>78</v>
@@ -2026,7 +2023,7 @@
         <v>84</v>
       </c>
       <c r="K18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M18" t="s">
         <v>78</v>
@@ -2035,7 +2032,7 @@
         <v>85</v>
       </c>
       <c r="O18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P18" t="s">
         <v>84</v>
@@ -2047,7 +2044,7 @@
         <v>85</v>
       </c>
       <c r="T18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U18" t="s">
         <v>89</v>
@@ -2059,7 +2056,7 @@
         <v>84</v>
       </c>
       <c r="Y18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Z18" t="s">
         <v>85</v>
@@ -2074,7 +2071,7 @@
         <v>78</v>
       </c>
       <c r="AE18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.45">
@@ -2085,7 +2082,7 @@
         <v>74</v>
       </c>
       <c r="C19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D19" t="s">
         <v>78</v>
@@ -2094,7 +2091,7 @@
         <v>85</v>
       </c>
       <c r="H19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I19" t="s">
         <v>78</v>
@@ -2103,7 +2100,7 @@
         <v>85</v>
       </c>
       <c r="M19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N19" t="s">
         <v>85</v>
@@ -2112,7 +2109,7 @@
         <v>78</v>
       </c>
       <c r="R19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S19" t="s">
         <v>78</v>
@@ -2124,7 +2121,7 @@
         <v>78</v>
       </c>
       <c r="X19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y19" t="s">
         <v>85</v>
@@ -2136,7 +2133,7 @@
         <v>78</v>
       </c>
       <c r="AD19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.45">
@@ -2147,7 +2144,7 @@
         <v>74</v>
       </c>
       <c r="C20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D20" t="s">
         <v>78</v>
@@ -2162,12 +2159,12 @@
         <v>78</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K20" s="30"/>
       <c r="L20" s="30"/>
       <c r="M20" s="30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N20" s="30" t="s">
         <v>85</v>
@@ -2184,7 +2181,7 @@
         <v>78</v>
       </c>
       <c r="T20" s="30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U20" s="30"/>
       <c r="V20" s="30"/>
@@ -2192,7 +2189,7 @@
         <v>78</v>
       </c>
       <c r="X20" s="30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y20" t="s">
         <v>85</v>
@@ -2219,7 +2216,7 @@
         <v>78</v>
       </c>
       <c r="F21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H21" t="s">
         <v>78</v>
@@ -2231,7 +2228,7 @@
         <v>84</v>
       </c>
       <c r="K21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M21" t="s">
         <v>78</v>
@@ -2243,13 +2240,13 @@
         <v>84</v>
       </c>
       <c r="P21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R21" t="s">
         <v>78</v>
       </c>
       <c r="S21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T21" t="s">
         <v>85</v>
@@ -2258,7 +2255,7 @@
         <v>84</v>
       </c>
       <c r="W21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X21" t="s">
         <v>89</v>
@@ -2276,7 +2273,7 @@
         <v>78</v>
       </c>
       <c r="AD21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE21" t="s">
         <v>85</v>
@@ -2290,7 +2287,7 @@
         <v>74</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D22" t="s">
         <v>78</v>
@@ -2305,7 +2302,7 @@
         <v>85</v>
       </c>
       <c r="O22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R22" t="s">
         <v>78</v>
@@ -2314,7 +2311,7 @@
         <v>85</v>
       </c>
       <c r="T22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W22" t="s">
         <v>78</v>
@@ -2323,10 +2320,10 @@
         <v>85</v>
       </c>
       <c r="Y22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC22" t="s">
         <v>78</v>
@@ -2343,7 +2340,7 @@
         <v>74</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D23" t="s">
         <v>78</v>
@@ -2358,19 +2355,19 @@
         <v>85</v>
       </c>
       <c r="J23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M23" t="s">
         <v>78</v>
       </c>
       <c r="N23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O23" t="s">
         <v>85</v>
       </c>
       <c r="R23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S23" t="s">
         <v>78</v>
@@ -2382,13 +2379,13 @@
         <v>85</v>
       </c>
       <c r="X23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y23" t="s">
         <v>78</v>
       </c>
       <c r="AB23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC23" t="s">
         <v>78</v>
@@ -2405,7 +2402,7 @@
         <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D24" t="s">
         <v>78</v>
@@ -2417,7 +2414,7 @@
         <v>85</v>
       </c>
       <c r="H24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I24" t="s">
         <v>78</v>
@@ -2429,7 +2426,7 @@
         <v>85</v>
       </c>
       <c r="M24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N24" t="s">
         <v>78</v>
@@ -2450,7 +2447,7 @@
         <v>78</v>
       </c>
       <c r="U24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W24" t="s">
         <v>89</v>
@@ -2462,7 +2459,7 @@
         <v>78</v>
       </c>
       <c r="Z24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB24" t="s">
         <v>86</v>
@@ -2471,7 +2468,7 @@
         <v>78</v>
       </c>
       <c r="AD24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE24" t="s">
         <v>85</v>
@@ -2494,7 +2491,7 @@
         <v>85</v>
       </c>
       <c r="F25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H25" t="s">
         <v>78</v>
@@ -2503,7 +2500,7 @@
         <v>84</v>
       </c>
       <c r="J25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K25" t="s">
         <v>85</v>
@@ -2518,7 +2515,7 @@
         <v>78</v>
       </c>
       <c r="P25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R25" t="s">
         <v>84</v>
@@ -2527,7 +2524,7 @@
         <v>78</v>
       </c>
       <c r="T25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U25" t="s">
         <v>85</v>
@@ -2536,7 +2533,7 @@
         <v>78</v>
       </c>
       <c r="X25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y25" t="s">
         <v>84</v>
@@ -2551,7 +2548,7 @@
         <v>85</v>
       </c>
       <c r="AD25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE25" t="s">
         <v>86</v>
@@ -2565,7 +2562,7 @@
         <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D26" t="s">
         <v>86</v>
@@ -2583,13 +2580,13 @@
         <v>84</v>
       </c>
       <c r="J26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K26" t="s">
         <v>85</v>
       </c>
       <c r="M26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N26" t="s">
         <v>78</v>
@@ -2607,7 +2604,7 @@
         <v>84</v>
       </c>
       <c r="T26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U26" t="s">
         <v>85</v>
@@ -2619,7 +2616,7 @@
         <v>78</v>
       </c>
       <c r="Y26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Z26" t="s">
         <v>86</v>
@@ -2634,7 +2631,7 @@
         <v>85</v>
       </c>
       <c r="AE26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.45">
@@ -2654,13 +2651,13 @@
         <v>86</v>
       </c>
       <c r="F27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H27" t="s">
         <v>85</v>
       </c>
       <c r="I27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J27" t="s">
         <v>84</v>
@@ -2672,7 +2669,7 @@
         <v>85</v>
       </c>
       <c r="N27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O27" t="s">
         <v>84</v>
@@ -2681,7 +2678,7 @@
         <v>78</v>
       </c>
       <c r="R27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S27" t="s">
         <v>84</v>
@@ -2696,7 +2693,7 @@
         <v>78</v>
       </c>
       <c r="AC27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD27" t="s">
         <v>86</v>
@@ -2716,7 +2713,7 @@
         <v>86</v>
       </c>
       <c r="D28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
         <v>85</v>
@@ -2725,7 +2722,7 @@
         <v>78</v>
       </c>
       <c r="M28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N28" t="s">
         <v>89</v>
@@ -2746,7 +2743,7 @@
         <v>89</v>
       </c>
       <c r="U28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W28" t="s">
         <v>89</v>
@@ -2755,7 +2752,7 @@
         <v>78</v>
       </c>
       <c r="Y28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Z28" t="s">
         <v>85</v>
@@ -2770,7 +2767,7 @@
         <v>85</v>
       </c>
       <c r="AE28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.45">
@@ -2784,7 +2781,7 @@
         <v>78</v>
       </c>
       <c r="D29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E29" t="s">
         <v>85</v>
@@ -2793,13 +2790,13 @@
         <v>85</v>
       </c>
       <c r="I29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J29" t="s">
         <v>78</v>
       </c>
       <c r="M29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N29" t="s">
         <v>85</v>
@@ -2808,7 +2805,7 @@
         <v>78</v>
       </c>
       <c r="W29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X29" t="s">
         <v>85</v>
@@ -2820,7 +2817,7 @@
         <v>85</v>
       </c>
       <c r="AC29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD29" t="s">
         <v>78</v>
@@ -2837,19 +2834,19 @@
         <v>78</v>
       </c>
       <c r="D30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W30" t="s">
         <v>78</v>
       </c>
       <c r="X30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB30" t="s">
         <v>78</v>
       </c>
       <c r="AC30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.45">
@@ -2863,13 +2860,13 @@
         <v>85</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E31" t="s">
         <v>78</v>
       </c>
       <c r="H31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I31" t="s">
         <v>85</v>
@@ -2884,19 +2881,19 @@
         <v>85</v>
       </c>
       <c r="O31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R31" t="s">
         <v>78</v>
       </c>
       <c r="S31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T31" t="s">
         <v>85</v>
       </c>
       <c r="W31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X31" t="s">
         <v>85</v>
@@ -2911,7 +2908,7 @@
         <v>85</v>
       </c>
       <c r="AD31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.45">
@@ -2928,7 +2925,7 @@
         <v>78</v>
       </c>
       <c r="E32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H32" t="s">
         <v>78</v>
@@ -2937,7 +2934,7 @@
         <v>85</v>
       </c>
       <c r="J32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M32" t="s">
         <v>78</v>
@@ -2946,10 +2943,10 @@
         <v>85</v>
       </c>
       <c r="O32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S32" t="s">
         <v>78</v>
@@ -2964,7 +2961,7 @@
         <v>78</v>
       </c>
       <c r="Y32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB32" s="29"/>
       <c r="AC32" s="29"/>
@@ -2985,7 +2982,7 @@
         <v>78</v>
       </c>
       <c r="E33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H33" t="s">
         <v>85</v>
@@ -2994,7 +2991,7 @@
         <v>78</v>
       </c>
       <c r="J33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M33" t="s">
         <v>85</v>
@@ -3003,7 +3000,7 @@
         <v>78</v>
       </c>
       <c r="O33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R33" t="s">
         <v>78</v>
@@ -3012,10 +3009,10 @@
         <v>85</v>
       </c>
       <c r="T33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X33" t="s">
         <v>78</v>
@@ -3030,7 +3027,7 @@
         <v>85</v>
       </c>
       <c r="AD33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.45">
@@ -3047,13 +3044,13 @@
         <v>86</v>
       </c>
       <c r="E34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F34" t="s">
         <v>78</v>
       </c>
       <c r="H34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I34" t="s">
         <v>78</v>
@@ -3074,7 +3071,7 @@
         <v>78</v>
       </c>
       <c r="P34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R34" t="s">
         <v>84</v>
@@ -3083,7 +3080,7 @@
         <v>78</v>
       </c>
       <c r="T34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U34" t="s">
         <v>85</v>
@@ -3098,7 +3095,7 @@
         <v>84</v>
       </c>
       <c r="Z34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB34" t="s">
         <v>85</v>
@@ -3107,7 +3104,7 @@
         <v>86</v>
       </c>
       <c r="AD34" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE34" t="s">
         <v>78</v>
@@ -3130,13 +3127,13 @@
         <v>78</v>
       </c>
       <c r="F35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H35" t="s">
         <v>78</v>
       </c>
       <c r="I35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J35" t="s">
         <v>85</v>
@@ -3154,7 +3151,7 @@
         <v>84</v>
       </c>
       <c r="P35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R35" t="s">
         <v>78</v>
@@ -3163,7 +3160,7 @@
         <v>84</v>
       </c>
       <c r="T35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U35" t="s">
         <v>85</v>
@@ -3175,7 +3172,7 @@
         <v>85</v>
       </c>
       <c r="Y35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Z35" t="s">
         <v>78</v>
@@ -3184,7 +3181,7 @@
         <v>86</v>
       </c>
       <c r="AC35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD35" t="s">
         <v>78</v>
@@ -3210,7 +3207,7 @@
         <v>86</v>
       </c>
       <c r="F36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M36" t="s">
         <v>85</v>
@@ -3222,7 +3219,7 @@
         <v>78</v>
       </c>
       <c r="P36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R36" t="s">
         <v>85</v>
@@ -3234,10 +3231,10 @@
         <v>84</v>
       </c>
       <c r="U36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X36" t="s">
         <v>86</v>
@@ -3255,10 +3252,10 @@
         <v>78</v>
       </c>
       <c r="AD36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE36" s="29" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.45">
@@ -3269,7 +3266,7 @@
         <v>74</v>
       </c>
       <c r="C37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D37" t="s">
         <v>85</v>
@@ -3284,13 +3281,13 @@
         <v>85</v>
       </c>
       <c r="J37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M37" t="s">
         <v>78</v>
       </c>
       <c r="N37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O37" t="s">
         <v>85</v>
@@ -3302,10 +3299,10 @@
         <v>85</v>
       </c>
       <c r="T37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X37" t="s">
         <v>78</v>
@@ -3317,7 +3314,7 @@
         <v>78</v>
       </c>
       <c r="AC37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD37" t="s">
         <v>85</v>
@@ -3337,7 +3334,7 @@
         <v>78</v>
       </c>
       <c r="E38" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB38" t="s">
         <v>85</v>
@@ -3346,7 +3343,7 @@
         <v>78</v>
       </c>
       <c r="AD38" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="39" spans="1:31" x14ac:dyDescent="0.45">
@@ -3360,7 +3357,7 @@
         <v>78</v>
       </c>
       <c r="D39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E39" t="s">
         <v>86</v>
@@ -3378,7 +3375,7 @@
         <v>85</v>
       </c>
       <c r="P39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R39" t="s">
         <v>85</v>
@@ -3387,7 +3384,7 @@
         <v>78</v>
       </c>
       <c r="T39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U39" t="s">
         <v>84</v>
@@ -3396,7 +3393,7 @@
         <v>78</v>
       </c>
       <c r="X39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y39" t="s">
         <v>85</v>
@@ -3411,7 +3408,7 @@
         <v>78</v>
       </c>
       <c r="AD39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE39" t="s">
         <v>86</v>
@@ -3434,7 +3431,7 @@
         <v>78</v>
       </c>
       <c r="F40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H40" t="s">
         <v>89</v>
@@ -3443,13 +3440,13 @@
         <v>78</v>
       </c>
       <c r="J40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K40" t="s">
         <v>85</v>
       </c>
       <c r="M40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N40" t="s">
         <v>84</v>
@@ -3467,7 +3464,7 @@
         <v>84</v>
       </c>
       <c r="T40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U40" t="s">
         <v>85</v>
@@ -3482,7 +3479,7 @@
         <v>89</v>
       </c>
       <c r="Z40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB40" t="s">
         <v>85</v>
@@ -3491,7 +3488,7 @@
         <v>78</v>
       </c>
       <c r="AD40" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE40" t="s">
         <v>86</v>
@@ -3511,13 +3508,13 @@
         <v>78</v>
       </c>
       <c r="E41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H41" t="s">
         <v>85</v>
       </c>
       <c r="I41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J41" t="s">
         <v>78</v>
@@ -3533,10 +3530,10 @@
         <v>78</v>
       </c>
       <c r="T41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X41" t="s">
         <v>85</v>
@@ -3545,7 +3542,7 @@
         <v>78</v>
       </c>
       <c r="AB41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AC41" t="s">
         <v>78</v>
@@ -3568,7 +3565,7 @@
         <v>78</v>
       </c>
       <c r="E42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H42" t="s">
         <v>85</v>
@@ -3577,7 +3574,7 @@
         <v>78</v>
       </c>
       <c r="J42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M42" t="s">
         <v>78</v>
@@ -3586,10 +3583,10 @@
         <v>85</v>
       </c>
       <c r="O42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="S42" t="s">
         <v>78</v>
@@ -3604,7 +3601,7 @@
         <v>85</v>
       </c>
       <c r="Y42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB42" t="s">
         <v>85</v>
@@ -3613,7 +3610,7 @@
         <v>78</v>
       </c>
       <c r="AD42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:31" x14ac:dyDescent="0.45">
@@ -3633,7 +3630,7 @@
         <v>78</v>
       </c>
       <c r="F43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H43" t="s">
         <v>85</v>
@@ -3645,7 +3642,7 @@
         <v>89</v>
       </c>
       <c r="K43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M43" t="s">
         <v>78</v>
@@ -3657,13 +3654,13 @@
         <v>85</v>
       </c>
       <c r="P43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R43" t="s">
         <v>85</v>
       </c>
       <c r="S43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="T43" t="s">
         <v>89</v>
@@ -3678,7 +3675,7 @@
         <v>85</v>
       </c>
       <c r="Y43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Z43" t="s">
         <v>86</v>
@@ -3693,7 +3690,7 @@
         <v>86</v>
       </c>
       <c r="AE43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:31" x14ac:dyDescent="0.45">
@@ -3707,7 +3704,7 @@
         <v>78</v>
       </c>
       <c r="D44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E44" t="s">
         <v>86</v>
@@ -3725,7 +3722,7 @@
         <v>78</v>
       </c>
       <c r="K44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M44" t="s">
         <v>78</v>
@@ -3734,7 +3731,7 @@
         <v>84</v>
       </c>
       <c r="O44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P44" t="s">
         <v>85</v>
@@ -3749,10 +3746,10 @@
         <v>84</v>
       </c>
       <c r="U44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="X44" t="s">
         <v>84</v>
@@ -3770,7 +3767,7 @@
         <v>78</v>
       </c>
       <c r="AD44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AE44" t="s">
         <v>85</v>
@@ -3796,7 +3793,7 @@
         <v>78</v>
       </c>
       <c r="G45" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H45" t="s">
         <v>84</v>
@@ -3808,7 +3805,7 @@
         <v>78</v>
       </c>
       <c r="K45" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L45" t="s">
         <v>89</v>
@@ -3826,7 +3823,7 @@
         <v>85</v>
       </c>
       <c r="Q45" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="R45" t="s">
         <v>84</v>
@@ -3835,7 +3832,7 @@
         <v>78</v>
       </c>
       <c r="T45" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="U45" t="s">
         <v>85</v>
@@ -3852,7 +3849,7 @@
         <v>74</v>
       </c>
       <c r="C46" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D46" s="29" t="s">
         <v>78</v>
@@ -3864,13 +3861,13 @@
         <v>78</v>
       </c>
       <c r="I46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J46" t="s">
         <v>85</v>
       </c>
       <c r="M46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N46" t="s">
         <v>78</v>
@@ -3885,7 +3882,7 @@
         <v>78</v>
       </c>
       <c r="T46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="W46" t="s">
         <v>78</v>
@@ -3894,13 +3891,13 @@
         <v>85</v>
       </c>
       <c r="Y46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AB46" t="s">
         <v>78</v>
       </c>
       <c r="AC46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AD46" t="s">
         <v>85</v>

</xml_diff>

<commit_message>
corrected mistakes from last commit
</commit_message>
<xml_diff>
--- a/data/hbsc_labels.xlsx
+++ b/data/hbsc_labels.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hanst\.rstudio\projects\Bechtiger &amp; Janousch (2025) Adolescent Well-Being in Flux\Adolescent-Well-Being-in-Flux\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uzh-my.sharepoint.com/personal/hansjoseph_thalathara_jacobscenter_uzh_ch/Documents/Datenanalyse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26099BAC-5934-499A-B312-E17E0238B5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{26099BAC-5934-499A-B312-E17E0238B5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29F1AB73-F4F7-4988-8B70-EC07AE02827E}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3255,7 +3255,7 @@
         <v>107</v>
       </c>
       <c r="AE36" s="29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.45">

</xml_diff>